<commit_message>
Resolve operating cost gaps
</commit_message>
<xml_diff>
--- a/08_Reports - Доклади - Berichte/Master_Financial_Timeline_Strict/master_financial_timeline_strict.xlsx
+++ b/08_Reports - Доклади - Berichte/Master_Financial_Timeline_Strict/master_financial_timeline_strict.xlsx
@@ -200,12 +200,12 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t/>
+          <t>20898.67</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t/>
+          <t>40.00</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -215,12 +215,12 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>18</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -230,7 +230,7 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Missing strict included values for: health insurance, operating cost; 12 excluded/unknown amount rows not summed</t>
+          <t>Missing strict included values for: health insurance; 13 excluded/unknown amount rows not summed</t>
         </is>
       </c>
     </row>
@@ -312,12 +312,12 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t/>
+          <t>18617.68</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t/>
+          <t>40.00</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -332,7 +332,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>14</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -342,7 +342,7 @@
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Missing strict included values for: health insurance, operating cost; 10 excluded/unknown amount rows not summed</t>
+          <t>Missing strict included values for: health insurance; 10 excluded/unknown amount rows not summed</t>
         </is>
       </c>
     </row>
@@ -424,12 +424,12 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t/>
+          <t>101.20</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t/>
+          <t>40.00</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -444,7 +444,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>11</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -454,7 +454,7 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>Missing strict included values for: health insurance, tax, operating cost; 8 excluded/unknown amount rows not summed</t>
+          <t>Missing strict included values for: health insurance, tax; 8 excluded/unknown amount rows not summed</t>
         </is>
       </c>
     </row>
@@ -536,12 +536,12 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t/>
+          <t>22955.19</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t/>
+          <t>40.00</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -556,7 +556,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>11</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -566,7 +566,7 @@
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>Missing strict included values for: payroll, health insurance, operating cost; 8 excluded/unknown amount rows not summed</t>
+          <t>Missing strict included values for: payroll, health insurance; 8 excluded/unknown amount rows not summed</t>
         </is>
       </c>
     </row>
@@ -648,12 +648,12 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t/>
+          <t>24058.49</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t/>
+          <t>40.00</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -668,7 +668,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>10</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -678,7 +678,7 @@
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>Missing strict included values for: payroll, health insurance, operating cost; 12 excluded/unknown amount rows not summed</t>
+          <t>Missing strict included values for: payroll, health insurance; 12 excluded/unknown amount rows not summed</t>
         </is>
       </c>
     </row>
@@ -760,12 +760,12 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t/>
+          <t>23553.36</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t/>
+          <t>40.00</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -780,7 +780,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>Missing strict included values for: payroll, operating cost; 8 excluded/unknown amount rows not summed</t>
+          <t>Missing strict included values for: payroll; 8 excluded/unknown amount rows not summed</t>
         </is>
       </c>
     </row>
@@ -872,12 +872,12 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t/>
+          <t>23067.09</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t/>
+          <t>40.00</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -892,7 +892,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -902,7 +902,7 @@
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>Missing strict included values for: operating cost; 9 excluded/unknown amount rows not summed</t>
+          <t>9 excluded/unknown amount rows not summed</t>
         </is>
       </c>
     </row>
@@ -984,12 +984,12 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t/>
+          <t>40.46</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t/>
+          <t>40.00</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1014,7 +1014,7 @@
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>Missing strict included values for: operating cost; 8 excluded/unknown amount rows not summed</t>
+          <t>8 excluded/unknown amount rows not summed</t>
         </is>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t/>
+          <t>22536.76</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
@@ -1116,7 +1116,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1126,7 +1126,7 @@
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>Missing strict included values for: payroll, operating cost; 4 excluded/unknown amount rows not summed</t>
+          <t>Missing strict included values for: payroll; 4 excluded/unknown amount rows not summed</t>
         </is>
       </c>
     </row>
@@ -1208,12 +1208,12 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t/>
+          <t>24246.81</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t/>
+          <t>40.00</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
@@ -1228,7 +1228,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>11</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>Missing strict included values for: operating cost; 9 excluded/unknown amount rows not summed</t>
+          <t>9 excluded/unknown amount rows not summed</t>
         </is>
       </c>
     </row>
@@ -1320,12 +1320,12 @@
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t/>
+          <t>27989.44</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t/>
+          <t>40.00</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
@@ -1340,7 +1340,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>18</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1350,7 +1350,7 @@
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>Missing strict included values for: payroll, operating cost; 12 excluded/unknown amount rows not summed</t>
+          <t>Missing strict included values for: payroll; 12 excluded/unknown amount rows not summed</t>
         </is>
       </c>
     </row>
@@ -1432,12 +1432,12 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t/>
+          <t>23984.73</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t/>
+          <t>40.00</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
@@ -1452,7 +1452,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>13</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1462,7 +1462,7 @@
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>Missing strict included values for: payroll, operating cost; 9 excluded/unknown amount rows not summed</t>
+          <t>Missing strict included values for: payroll; 9 excluded/unknown amount rows not summed</t>
         </is>
       </c>
     </row>
@@ -1544,7 +1544,7 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t/>
+          <t>24159.32</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
@@ -1564,7 +1564,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1574,7 +1574,7 @@
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>Missing strict included values for: payroll, operating cost; 5 excluded/unknown amount rows not summed</t>
+          <t>Missing strict included values for: payroll; 5 excluded/unknown amount rows not summed</t>
         </is>
       </c>
     </row>
@@ -1656,7 +1656,7 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t/>
+          <t>22523.36</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
@@ -1676,7 +1676,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -1686,7 +1686,7 @@
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>Missing strict included values for: payroll, operating cost; 4 excluded/unknown amount rows not summed</t>
+          <t>Missing strict included values for: payroll; 4 excluded/unknown amount rows not summed</t>
         </is>
       </c>
     </row>
@@ -1773,7 +1773,7 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t/>
+          <t>80.00</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -1783,14 +1783,14 @@
       </c>
       <c r="S16" t="inlineStr">
         <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
           <t>15</t>
         </is>
       </c>
-      <c r="T16" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
       <c r="U16" t="inlineStr">
         <is>
           <t>MEDIUM</t>
@@ -1798,7 +1798,7 @@
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>Missing strict included values for: payroll, health insurance, operating cost; 15 excluded/unknown amount rows not summed</t>
+          <t>Missing strict included values for: payroll, health insurance; 16 excluded/unknown amount rows not summed</t>
         </is>
       </c>
     </row>

</xml_diff>